<commit_message>
Help function random baseline
+ changed data to test
</commit_message>
<xml_diff>
--- a/data/raw_data/school_1/OpzetDataAnoniem.xlsx
+++ b/data/raw_data/school_1/OpzetDataAnoniem.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amber/Desktop/Scriptie/Master/OpzetData/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amber/Desktop/Thesis/data/raw_data/school_1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25FBA35E-E9C9-1B4A-8CDF-E1856E9E061F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CA199EC-7432-1E44-BB88-AB2C96234A11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="15520" activeTab="4" xr2:uid="{74F643B1-BB2A-D446-89B2-FA7548F43674}"/>
+    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="15520" activeTab="2" xr2:uid="{74F643B1-BB2A-D446-89B2-FA7548F43674}"/>
   </bookViews>
   <sheets>
     <sheet name="UITLEG" sheetId="9" r:id="rId1"/>
@@ -626,7 +626,13 @@
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{757CC562-ADFC-1E47-ACD2-2B6F988CB029}" name="Table5" displayName="Table5" ref="A2:J117">
-  <autoFilter ref="A2:J117" xr:uid="{757CC562-ADFC-1E47-ACD2-2B6F988CB029}"/>
+  <autoFilter ref="A2:J117" xr:uid="{757CC562-ADFC-1E47-ACD2-2B6F988CB029}">
+    <filterColumn colId="4">
+      <filters blank="1">
+        <filter val="Ja"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{7DE3C0FB-F63C-0442-99D4-615EC68F9FF0}" name="Naam leerling" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{22FD41B5-871F-294E-906A-CC31EDC5EB0A}" name="Nieuwe groep"/>
@@ -1267,7 +1273,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>57</v>
       </c>
@@ -1299,7 +1305,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>58</v>
       </c>
@@ -1331,7 +1337,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>59</v>
       </c>
@@ -1363,7 +1369,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>60</v>
       </c>
@@ -1427,7 +1433,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>62</v>
       </c>
@@ -1459,7 +1465,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>63</v>
       </c>
@@ -1491,7 +1497,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>64</v>
       </c>
@@ -1523,7 +1529,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>65</v>
       </c>
@@ -1587,7 +1593,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>67</v>
       </c>
@@ -1619,7 +1625,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>68</v>
       </c>
@@ -1651,7 +1657,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>69</v>
       </c>
@@ -1715,7 +1721,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>71</v>
       </c>
@@ -1747,7 +1753,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>72</v>
       </c>
@@ -1779,7 +1785,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>73</v>
       </c>
@@ -1811,7 +1817,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>74</v>
       </c>
@@ -1843,7 +1849,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>75</v>
       </c>
@@ -1875,7 +1881,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>76</v>
       </c>
@@ -1907,7 +1913,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>77</v>
       </c>
@@ -1939,7 +1945,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>78</v>
       </c>
@@ -1971,7 +1977,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>79</v>
       </c>
@@ -2067,7 +2073,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>82</v>
       </c>
@@ -2099,7 +2105,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>83</v>
       </c>
@@ -2131,7 +2137,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>84</v>
       </c>
@@ -2163,7 +2169,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>85</v>
       </c>
@@ -2245,7 +2251,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>56</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -2261,7 +2267,7 @@
         <v>0</v>
       </c>
       <c r="B5">
-        <v>25</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -2269,7 +2275,7 @@
         <v>20</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -2277,7 +2283,7 @@
         <v>21</v>
       </c>
       <c r="B7">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added random baseline to pipeline
+ moved data validation to separate file
</commit_message>
<xml_diff>
--- a/data/raw_data/school_1/OpzetDataAnoniem.xlsx
+++ b/data/raw_data/school_1/OpzetDataAnoniem.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amber/Desktop/Thesis/data/raw_data/school_1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CA199EC-7432-1E44-BB88-AB2C96234A11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6483A764-435C-5F4C-9CB2-1B1D1567303E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="15520" activeTab="2" xr2:uid="{74F643B1-BB2A-D446-89B2-FA7548F43674}"/>
+    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="15520" activeTab="1" xr2:uid="{74F643B1-BB2A-D446-89B2-FA7548F43674}"/>
   </bookViews>
   <sheets>
     <sheet name="UITLEG" sheetId="9" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="89">
   <si>
     <t>Minimale groepsgrootte</t>
   </si>
@@ -344,9 +344,6 @@
   </si>
   <si>
     <t>Docent3</t>
-  </si>
-  <si>
-    <t>Docent4</t>
   </si>
   <si>
     <t>Docent5</t>
@@ -1140,7 +1137,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0132EB3-FD4E-104A-B4EA-93080333F476}">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.5" customWidth="1"/>
@@ -1170,16 +1167,6 @@
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>53</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1243,962 +1230,962 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B3">
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" t="s">
         <v>88</v>
       </c>
-      <c r="E3" t="s">
-        <v>89</v>
-      </c>
       <c r="F3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B4">
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B6">
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B7">
         <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B8">
         <v>4</v>
       </c>
       <c r="C8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D8" t="s">
+        <v>87</v>
+      </c>
+      <c r="E8" t="s">
         <v>88</v>
       </c>
-      <c r="E8" t="s">
-        <v>89</v>
-      </c>
       <c r="F8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B9">
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B10">
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B11">
         <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B12">
         <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B13">
         <v>4</v>
       </c>
       <c r="C13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D13" t="s">
+        <v>87</v>
+      </c>
+      <c r="E13" t="s">
         <v>88</v>
       </c>
-      <c r="E13" t="s">
-        <v>89</v>
-      </c>
       <c r="F13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G13" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H13" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B14">
         <v>4</v>
       </c>
       <c r="C14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B15">
         <v>4</v>
       </c>
       <c r="C15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D15" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E15" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B16">
         <v>4</v>
       </c>
       <c r="C16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D16" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E16" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B17">
         <v>4</v>
       </c>
       <c r="C17" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D17" t="s">
+        <v>87</v>
+      </c>
+      <c r="E17" t="s">
         <v>88</v>
       </c>
-      <c r="E17" t="s">
-        <v>89</v>
-      </c>
       <c r="F17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H17" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B18">
         <v>4</v>
       </c>
       <c r="C18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D18" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E18" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F18" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I18" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B19">
         <v>4</v>
       </c>
       <c r="C19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D19" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E19" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G19" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H19" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J19" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B20">
         <v>4</v>
       </c>
       <c r="C20" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D20" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E20" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I20" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B21">
         <v>4</v>
       </c>
       <c r="C21" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D21" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E21" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F21" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G21" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H21" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I21" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J21" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B22">
         <v>4</v>
       </c>
       <c r="C22" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D22" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E22" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H22" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J22" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B23">
         <v>5</v>
       </c>
       <c r="C23" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D23" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E23" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F23" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I23" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J23" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B24">
         <v>5</v>
       </c>
       <c r="C24" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D24" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E24" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F24" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G24" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H24" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I24" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J24" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B25">
         <v>5</v>
       </c>
       <c r="C25" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F25" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J25" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B26">
         <v>5</v>
       </c>
       <c r="C26" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D26" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E26" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G26" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I26" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B27">
         <v>5</v>
       </c>
       <c r="C27" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D27" t="s">
+        <v>87</v>
+      </c>
+      <c r="E27" t="s">
         <v>88</v>
       </c>
-      <c r="E27" t="s">
-        <v>89</v>
-      </c>
       <c r="F27" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G27" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J27" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B28">
         <v>5</v>
       </c>
       <c r="C28" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D28" t="s">
+        <v>87</v>
+      </c>
+      <c r="E28" t="s">
         <v>88</v>
       </c>
-      <c r="E28" t="s">
-        <v>89</v>
-      </c>
       <c r="F28" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H28" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I28" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J28" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B29">
         <v>5</v>
       </c>
       <c r="C29" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D29" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E29" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F29" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G29" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H29" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I29" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J29" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="30" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B30">
         <v>5</v>
       </c>
       <c r="C30" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D30" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E30" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G30" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H30" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I30" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J30" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B31">
         <v>5</v>
       </c>
       <c r="C31" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D31" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E31" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F31" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H31" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I31" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J31" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B32">
         <v>5</v>
       </c>
       <c r="C32" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D32" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E32" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F32" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G32" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H32" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I32" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J32" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -2304,46 +2291,46 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C12" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
@@ -2364,46 +2351,46 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B24" t="s">
         <v>53</v>
       </c>
       <c r="C24" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B25" t="s">
         <v>52</v>
       </c>
       <c r="C25" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B26" t="s">
         <v>53</v>
       </c>
       <c r="C26" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B27" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C27" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -2461,7 +2448,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
         <v>51</v>
@@ -2469,7 +2456,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B4" t="s">
         <v>51</v>
@@ -2477,7 +2464,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B5" t="s">
         <v>51</v>
@@ -2485,7 +2472,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B6" t="s">
         <v>51</v>
@@ -2493,7 +2480,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B7" t="s">
         <v>51</v>
@@ -2501,7 +2488,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B8" t="s">
         <v>51</v>
@@ -2509,7 +2496,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B9" t="s">
         <v>51</v>
@@ -2517,7 +2504,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B10" t="s">
         <v>51</v>
@@ -2525,7 +2512,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B11" t="s">
         <v>51</v>
@@ -2533,7 +2520,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B12" t="s">
         <v>51</v>
@@ -2541,7 +2528,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B13" t="s">
         <v>51</v>
@@ -2549,7 +2536,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B14" t="s">
         <v>51</v>
@@ -2557,7 +2544,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B15" t="s">
         <v>51</v>
@@ -2565,7 +2552,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B16" t="s">
         <v>51</v>
@@ -2573,7 +2560,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B17" t="s">
         <v>51</v>
@@ -2581,7 +2568,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B18" t="s">
         <v>52</v>
@@ -2589,7 +2576,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B19" t="s">
         <v>53</v>
@@ -2597,31 +2584,31 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B23" t="s">
         <v>52</v>
@@ -2629,7 +2616,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B24" t="s">
         <v>51</v>
@@ -2637,15 +2624,15 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B25" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B26" t="s">
         <v>52</v>
@@ -2653,7 +2640,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B27" t="s">
         <v>52</v>
@@ -2661,7 +2648,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B28" t="s">
         <v>52</v>
@@ -2669,7 +2656,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B29" t="s">
         <v>52</v>
@@ -2677,7 +2664,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B30" t="s">
         <v>52</v>
@@ -2685,7 +2672,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B31" t="s">
         <v>52</v>
@@ -2693,7 +2680,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B32" t="s">
         <v>52</v>

</xml_diff>

<commit_message>
MILP model that returns infeasible
</commit_message>
<xml_diff>
--- a/data/raw_data/school_1/OpzetDataAnoniem.xlsx
+++ b/data/raw_data/school_1/OpzetDataAnoniem.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amber/Desktop/Thesis/data/raw_data/school_1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6483A764-435C-5F4C-9CB2-1B1D1567303E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8EEF835-9760-1143-9A55-D279BFCA15E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="15520" activeTab="1" xr2:uid="{74F643B1-BB2A-D446-89B2-FA7548F43674}"/>
+    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="15520" activeTab="4" xr2:uid="{74F643B1-BB2A-D446-89B2-FA7548F43674}"/>
   </bookViews>
   <sheets>
     <sheet name="UITLEG" sheetId="9" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="88">
   <si>
     <t>Minimale groepsgrootte</t>
   </si>
@@ -344,9 +344,6 @@
   </si>
   <si>
     <t>Docent3</t>
-  </si>
-  <si>
-    <t>Docent5</t>
   </si>
   <si>
     <t>Leerling1</t>
@@ -1230,962 +1227,962 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B3">
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E3" t="s">
         <v>87</v>
       </c>
-      <c r="E3" t="s">
-        <v>88</v>
-      </c>
       <c r="F3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B4">
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B6">
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B7">
         <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B8">
         <v>4</v>
       </c>
       <c r="C8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D8" t="s">
+        <v>86</v>
+      </c>
+      <c r="E8" t="s">
         <v>87</v>
       </c>
-      <c r="E8" t="s">
-        <v>88</v>
-      </c>
       <c r="F8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B9">
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B10">
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B11">
         <v>4</v>
       </c>
       <c r="C11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B12">
         <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B13">
         <v>4</v>
       </c>
       <c r="C13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D13" t="s">
+        <v>86</v>
+      </c>
+      <c r="E13" t="s">
         <v>87</v>
       </c>
-      <c r="E13" t="s">
-        <v>88</v>
-      </c>
       <c r="F13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B14">
         <v>4</v>
       </c>
       <c r="C14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H14" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B15">
         <v>4</v>
       </c>
       <c r="C15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B16">
         <v>4</v>
       </c>
       <c r="C16" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H16" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I16" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J16" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B17">
         <v>4</v>
       </c>
       <c r="C17" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D17" t="s">
+        <v>86</v>
+      </c>
+      <c r="E17" t="s">
         <v>87</v>
       </c>
-      <c r="E17" t="s">
-        <v>88</v>
-      </c>
       <c r="F17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H17" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I17" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J17" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B18">
         <v>4</v>
       </c>
       <c r="C18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D18" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F18" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B19">
         <v>4</v>
       </c>
       <c r="C19" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F19" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G19" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H19" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I19" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B20">
         <v>4</v>
       </c>
       <c r="C20" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D20" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E20" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I20" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J20" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="21" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B21">
         <v>4</v>
       </c>
       <c r="C21" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D21" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E21" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H21" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I21" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J21" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="22" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B22">
         <v>4</v>
       </c>
       <c r="C22" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D22" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E22" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H22" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I22" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J22" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B23">
         <v>5</v>
       </c>
       <c r="C23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D23" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E23" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F23" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B24">
         <v>5</v>
       </c>
       <c r="C24" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D24" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E24" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F24" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G24" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H24" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I24" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J24" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B25">
         <v>5</v>
       </c>
       <c r="C25" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D25" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E25" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F25" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H25" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J25" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B26">
         <v>5</v>
       </c>
       <c r="C26" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D26" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E26" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H26" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I26" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J26" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B27">
         <v>5</v>
       </c>
       <c r="C27" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D27" t="s">
+        <v>86</v>
+      </c>
+      <c r="E27" t="s">
         <v>87</v>
       </c>
-      <c r="E27" t="s">
-        <v>88</v>
-      </c>
       <c r="F27" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H27" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I27" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J27" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B28">
         <v>5</v>
       </c>
       <c r="C28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D28" t="s">
+        <v>86</v>
+      </c>
+      <c r="E28" t="s">
         <v>87</v>
       </c>
-      <c r="E28" t="s">
-        <v>88</v>
-      </c>
       <c r="F28" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H28" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I28" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J28" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B29">
         <v>5</v>
       </c>
       <c r="C29" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D29" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E29" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F29" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G29" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H29" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I29" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J29" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="30" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B30">
         <v>5</v>
       </c>
       <c r="C30" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D30" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E30" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F30" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I30" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J30" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B31">
         <v>5</v>
       </c>
       <c r="C31" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D31" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E31" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F31" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G31" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H31" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I31" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J31" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B32">
         <v>5</v>
       </c>
       <c r="C32" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D32" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E32" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F32" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G32" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H32" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I32" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J32" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -2291,46 +2288,46 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
@@ -2351,46 +2348,46 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B24" t="s">
         <v>53</v>
       </c>
       <c r="C24" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B25" t="s">
         <v>52</v>
       </c>
       <c r="C25" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B26" t="s">
         <v>53</v>
       </c>
       <c r="C26" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B27" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C27" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -2448,7 +2445,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
         <v>51</v>
@@ -2456,7 +2453,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B4" t="s">
         <v>51</v>
@@ -2464,7 +2461,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B5" t="s">
         <v>51</v>
@@ -2472,7 +2469,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
         <v>51</v>
@@ -2480,7 +2477,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B7" t="s">
         <v>51</v>
@@ -2488,7 +2485,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B8" t="s">
         <v>51</v>
@@ -2496,7 +2493,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B9" t="s">
         <v>51</v>
@@ -2504,7 +2501,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B10" t="s">
         <v>51</v>
@@ -2512,7 +2509,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B11" t="s">
         <v>51</v>
@@ -2520,7 +2517,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B12" t="s">
         <v>51</v>
@@ -2528,7 +2525,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B13" t="s">
         <v>51</v>
@@ -2536,7 +2533,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B14" t="s">
         <v>51</v>
@@ -2544,7 +2541,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B15" t="s">
         <v>51</v>
@@ -2552,7 +2549,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B16" t="s">
         <v>51</v>
@@ -2560,7 +2557,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B17" t="s">
         <v>51</v>
@@ -2568,7 +2565,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B18" t="s">
         <v>52</v>
@@ -2576,7 +2573,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B19" t="s">
         <v>53</v>
@@ -2584,7 +2581,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B20" t="s">
         <v>53</v>
@@ -2592,7 +2589,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B21" t="s">
         <v>53</v>
@@ -2600,7 +2597,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B22" t="s">
         <v>53</v>
@@ -2608,7 +2605,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B23" t="s">
         <v>52</v>
@@ -2616,7 +2613,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B24" t="s">
         <v>51</v>
@@ -2624,7 +2621,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B25" t="s">
         <v>53</v>
@@ -2632,7 +2629,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B26" t="s">
         <v>52</v>
@@ -2640,7 +2637,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B27" t="s">
         <v>52</v>
@@ -2648,7 +2645,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B28" t="s">
         <v>52</v>
@@ -2656,7 +2653,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B29" t="s">
         <v>52</v>
@@ -2664,7 +2661,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B30" t="s">
         <v>52</v>
@@ -2672,7 +2669,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B31" t="s">
         <v>52</v>
@@ -2680,7 +2677,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B32" t="s">
         <v>52</v>

</xml_diff>